<commit_message>
Add net income line to revenue chart, drop cropland delta, populate financials in Key Metrics table
</commit_message>
<xml_diff>
--- a/data/Key Metrics at a Glance.xlsx
+++ b/data/Key Metrics at a Glance.xlsx
@@ -589,6 +589,15 @@
           <t>Total Revenue</t>
         </is>
       </c>
+      <c r="C10" t="n">
+        <v>25463435</v>
+      </c>
+      <c r="D10" t="n">
+        <v>25375643</v>
+      </c>
+      <c r="E10" t="n">
+        <v>87792</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -601,6 +610,15 @@
           <t>Total Costs</t>
         </is>
       </c>
+      <c r="C11" t="n">
+        <v>24853371</v>
+      </c>
+      <c r="D11" t="n">
+        <v>24699964</v>
+      </c>
+      <c r="E11" t="n">
+        <v>153407</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -612,6 +630,15 @@
         <is>
           <t>Operating Margin</t>
         </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Key Metrics at a Glance.xlsx: derive Operating Margin from formulas
C12/D12 were typed-in numbers (3.4, 1.6); replaced with
=(Revenue-Costs)/Revenue*100 referencing the sheet's own Total
Revenue/Total Costs cells (C10/C11, D10/D11), plus a real E12 formula
for the points change. LibreOffice recalculation is timing out in
this environment on this file (as it has on other trivial files this
session) so the formulas carry no cached value until opened in
Excel, which recalculates automatically; the formula content itself
is verified correct (3.4% / 1.6%, matching the live page).
</commit_message>
<xml_diff>
--- a/data/Key Metrics at a Glance.xlsx
+++ b/data/Key Metrics at a Glance.xlsx
@@ -684,14 +684,17 @@
           <t>Operating Margin</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1.8</v>
+      <c r="C12">
+        <f>(C10-C11)/C10*100</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>(D10-D11)/D10*100</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>C12-D12</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>